<commit_message>
Versjon 2.5.5 · 7,5 % rente på banklån, nye Nordlys-tall i kap. 1, 3, 4, 6, 9, 12, 13 og markedsføring 3 og 10, Verktøy og måleinstrumenter
</commit_message>
<xml_diff>
--- a/pensum/ok01/OK01_Etablering_og_oppstart_Regneark_Selskapsform_og_skatt.xlsx
+++ b/pensum/ok01/OK01_Etablering_og_oppstart_Regneark_Selskapsform_og_skatt.xlsx
@@ -1065,12 +1065,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1078,11 +1082,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1090,7 +1094,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1098,11 +1102,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1110,7 +1114,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1122,31 +1126,31 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1154,71 +1158,71 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1486,207 +1490,207 @@
   <dimension ref="A1:C27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="7" t="n">
         <v>2400000</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="8" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="9" t="n">
         <v>0.5</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="8" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="7" t="n">
         <v>800000</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="8" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B8" s="7" t="n">
         <v>300000</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="8" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="10" t="n">
         <f aca="false">B5</f>
         <v>2400000</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="10" t="n">
         <f aca="false">B5</f>
         <v>2400000</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="9" t="n">
+      <c r="B13" s="10" t="n">
         <f aca="false">B5*B6</f>
         <v>1200000</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="8" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="10" t="n">
         <f aca="false">0*B5</f>
         <v>0</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="8" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="16" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="11" t="n">
+      <c r="B16" s="12" t="n">
         <f aca="false">B7+B8</f>
         <v>1100000</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="8" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B17" s="9" t="n">
+      <c r="B17" s="10" t="n">
         <f aca="false">B11-B16</f>
         <v>1300000</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="8" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12" t="str">
+      <c r="A20" s="13" t="str">
         <f aca="false">"I et enkeltpersonforetak skylder eieren "&amp;TEXT(ROUND(B11,0),"#,##0")&amp;" kroner. I et AS med kausjon kan eierne tape "&amp;TEXT(ROUND(B16,0),"#,##0")&amp;" kroner privat."</f>
         <v>I et enkeltpersonforetak skylder eieren 2,400,000 kroner. I et AS med kausjon kan eierne tape 1,100,000 kroner privat.</v>
       </c>
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="13" t="s">
+      <c r="A23" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="14"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="27" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
+      <c r="A27" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1715,302 +1719,302 @@
   <dimension ref="A1:C50"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="64"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="15" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="16" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="19" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="16" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="17" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="19" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="19" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="19" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="19" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="16" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="15" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="16" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="15" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="16" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="15" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="16" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="15" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="16" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="16" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="16" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="17" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="18" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="B25" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="C25" s="18" t="s">
+      <c r="C25" s="19" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="16" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="17" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="21" t="s">
+      <c r="A28" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="B28" s="21" t="s">
+      <c r="B28" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="C28" s="21" t="s">
+      <c r="C28" s="22" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="18" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="B29" s="20" t="s">
+      <c r="B29" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C29" s="18" t="s">
+      <c r="C29" s="19" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="18" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="B30" s="20" t="s">
+      <c r="B30" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C30" s="18" t="s">
+      <c r="C30" s="19" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="18" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="B31" s="20" t="s">
+      <c r="B31" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="C31" s="18" t="s">
+      <c r="C31" s="19" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="18" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="B32" s="20" t="s">
+      <c r="B32" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C32" s="18" t="s">
+      <c r="C32" s="19" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="18" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="B33" s="20" t="s">
+      <c r="B33" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="C33" s="18" t="s">
+      <c r="C33" s="19" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="18" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="B34" s="20" t="s">
+      <c r="B34" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="C34" s="18" t="s">
+      <c r="C34" s="19" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="18" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="B35" s="20" t="s">
+      <c r="B35" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C35" s="18" t="s">
+      <c r="C35" s="19" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="18" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="B36" s="20" t="s">
+      <c r="B36" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="C36" s="18" t="s">
+      <c r="C36" s="19" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="16" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="17" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="18" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="19" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="18" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="19" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="15" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="16" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="16" t="s">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="17" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="18" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="19" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="16" t="s">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="17" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="15" t="s">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="16" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="15" t="s">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="16" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="15" t="s">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="16" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="15" t="s">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="16" t="s">
         <v>91</v>
       </c>
     </row>
@@ -2033,388 +2037,388 @@
   <dimension ref="A1:F40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="54"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="15" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="21" t="s">
         <v>95</v>
       </c>
-      <c r="B5" s="22" t="n">
+      <c r="B5" s="23" t="n">
         <v>900000</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="19" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="B6" s="23" t="n">
+      <c r="B6" s="24" t="n">
         <v>0.34</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="19" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="B7" s="23" t="n">
+      <c r="B7" s="24" t="n">
         <v>0.22</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="19" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="B8" s="24" t="n">
+      <c r="B8" s="25" t="n">
         <v>1.72</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="B9" s="25" t="n">
+      <c r="B9" s="26" t="n">
         <f aca="false">B7*B8</f>
         <v>0.3784</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="19" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21"/>
-      <c r="B11" s="21" t="s">
+      <c r="A11" s="22"/>
+      <c r="B11" s="22" t="s">
         <v>104</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="D11" s="21" t="s">
+      <c r="D11" s="22" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="B12" s="26" t="n">
+      <c r="B12" s="27" t="n">
         <f aca="false">$B$5</f>
         <v>900000</v>
       </c>
-      <c r="C12" s="26" t="n">
+      <c r="C12" s="27" t="n">
         <f aca="false">$B$5</f>
         <v>900000</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="D12" s="19" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="26" t="n">
+      <c r="B13" s="27" t="n">
         <f aca="false">B12*$B$6</f>
         <v>306000</v>
       </c>
-      <c r="C13" s="26" t="n">
+      <c r="C13" s="27" t="n">
         <f aca="false">C12*$B$7</f>
         <v>198000</v>
       </c>
-      <c r="D13" s="18" t="s">
+      <c r="D13" s="19" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="B14" s="27" t="n">
+      <c r="B14" s="28" t="n">
         <f aca="false">B12-B13</f>
         <v>594000</v>
       </c>
-      <c r="C14" s="27" t="n">
+      <c r="C14" s="28" t="n">
         <f aca="false">C12-C13</f>
         <v>702000</v>
       </c>
-      <c r="D14" s="18" t="s">
+      <c r="D14" s="19" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="18" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="D15" s="18" t="s">
+      <c r="D15" s="19" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21" t="s">
         <v>116</v>
       </c>
-      <c r="C16" s="27" t="n">
+      <c r="C16" s="28" t="n">
         <f aca="false">C14-B14</f>
         <v>108000</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="19" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="16" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="17" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="18" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="C19" s="26" t="n">
+      <c r="C19" s="27" t="n">
         <f aca="false">C14*$B$9</f>
         <v>265636.8</v>
       </c>
-      <c r="D19" s="18" t="s">
+      <c r="D19" s="19" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="20" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="B20" s="27" t="n">
+      <c r="B20" s="28" t="n">
         <f aca="false">B14</f>
         <v>594000</v>
       </c>
-      <c r="C20" s="27" t="n">
+      <c r="C20" s="28" t="n">
         <f aca="false">C14-C19</f>
         <v>436363.2</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="D20" s="19" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="20" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="B21" s="28" t="n">
+      <c r="B21" s="29" t="n">
         <f aca="false">1-B20/$B$5</f>
         <v>0.34</v>
       </c>
-      <c r="C21" s="28" t="n">
+      <c r="C21" s="29" t="n">
         <f aca="false">1-C20/$B$5</f>
         <v>0.515152</v>
       </c>
-      <c r="D21" s="18" t="s">
+      <c r="D21" s="19" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="20" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="C22" s="27" t="n">
+      <c r="C22" s="28" t="n">
         <f aca="false">C20-B20</f>
         <v>-157636.8</v>
       </c>
-      <c r="D22" s="18" t="s">
+      <c r="D22" s="19" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="16" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="17" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="21" t="s">
+      <c r="A25" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="C25" s="21" t="s">
+      <c r="C25" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="D25" s="21" t="s">
+      <c r="D25" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="E25" s="21" t="s">
+      <c r="E25" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="F25" s="21" t="s">
+      <c r="F25" s="22" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="22" t="n">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="23" t="n">
         <v>300000</v>
       </c>
-      <c r="B26" s="26" t="n">
+      <c r="B26" s="27" t="n">
         <f aca="false">A26*(1-$B$6)</f>
         <v>198000</v>
       </c>
-      <c r="C26" s="26" t="n">
+      <c r="C26" s="27" t="n">
         <f aca="false">A26*(1-$B$7)</f>
         <v>234000</v>
       </c>
-      <c r="D26" s="26" t="n">
+      <c r="D26" s="27" t="n">
         <f aca="false">C26*(1-$B$9)</f>
         <v>145454.4</v>
       </c>
-      <c r="E26" s="26" t="n">
+      <c r="E26" s="27" t="n">
         <f aca="false">C26-B26</f>
         <v>36000</v>
       </c>
-      <c r="F26" s="26" t="n">
+      <c r="F26" s="27" t="n">
         <f aca="false">D26-B26</f>
         <v>-52545.6</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="22" t="n">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="23" t="n">
         <v>900000</v>
       </c>
-      <c r="B27" s="26" t="n">
+      <c r="B27" s="27" t="n">
         <f aca="false">A27*(1-$B$6)</f>
         <v>594000</v>
       </c>
-      <c r="C27" s="26" t="n">
+      <c r="C27" s="27" t="n">
         <f aca="false">A27*(1-$B$7)</f>
         <v>702000</v>
       </c>
-      <c r="D27" s="26" t="n">
+      <c r="D27" s="27" t="n">
         <f aca="false">C27*(1-$B$9)</f>
         <v>436363.2</v>
       </c>
-      <c r="E27" s="26" t="n">
+      <c r="E27" s="27" t="n">
         <f aca="false">C27-B27</f>
         <v>108000</v>
       </c>
-      <c r="F27" s="26" t="n">
+      <c r="F27" s="27" t="n">
         <f aca="false">D27-B27</f>
         <v>-157636.8</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="22" t="n">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="23" t="n">
         <v>1800000</v>
       </c>
-      <c r="B28" s="26" t="n">
+      <c r="B28" s="27" t="n">
         <f aca="false">A28*(1-$B$6)</f>
         <v>1188000</v>
       </c>
-      <c r="C28" s="26" t="n">
+      <c r="C28" s="27" t="n">
         <f aca="false">A28*(1-$B$7)</f>
         <v>1404000</v>
       </c>
-      <c r="D28" s="26" t="n">
+      <c r="D28" s="27" t="n">
         <f aca="false">C28*(1-$B$9)</f>
         <v>872726.4</v>
       </c>
-      <c r="E28" s="26" t="n">
+      <c r="E28" s="27" t="n">
         <f aca="false">C28-B28</f>
         <v>216000</v>
       </c>
-      <c r="F28" s="26" t="n">
+      <c r="F28" s="27" t="n">
         <f aca="false">D28-B28</f>
         <v>-315273.6</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="20" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="21" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="16" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="17" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="18" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="19" t="s">
         <v>137</v>
       </c>
-      <c r="B32" s="29" t="str">
+      <c r="B32" s="30" t="str">
         <f aca="false">IF(C16&gt;0,"OK — aksjeselskapet beholder mer av overskuddet så lenge pengene blir stående i selskapet","AVVIK: med disse satsene er det ingen skattefordel ved aksjeselskap i det hele tatt")</f>
         <v>OK — aksjeselskapet beholder mer av overskuddet så lenge pengene blir stående i selskapet</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="18" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="19" t="s">
         <v>138</v>
       </c>
-      <c r="B33" s="29" t="str">
+      <c r="B33" s="30" t="str">
         <f aca="false">IF(C22&lt;0,"OK — tar du alt ut, betaler du mer i aksjeselskap enn i enkeltpersonforetak. Det er kapitlets viktigste skattepoeng","AVVIK: sjekk satsene i B6, B7 og B8 — poenget i oppgave 2 forutsetter at fullt uttak er dyrere i aksjeselskap")</f>
         <v>OK — tar du alt ut, betaler du mer i aksjeselskap enn i enkeltpersonforetak. Det er kapitlets viktigste skattepoeng</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="18" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="B34" s="29" t="str">
+      <c r="B34" s="30" t="str">
         <f aca="false">IF(AND(ABS(B13+B14-B12)&lt;1,ABS(C13+C14-C12)&lt;1),"OK — skatt pluss rest er lik overskuddet i begge former","AVVIK: regnestykket går ikke opp")</f>
         <v>OK — skatt pluss rest er lik overskuddet i begge former</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="16" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="17" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="18" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="19" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="18" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="19" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="20" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="21" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="15" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="16" t="s">
         <v>144</v>
       </c>
     </row>
@@ -2452,221 +2456,221 @@
   <dimension ref="A1:C28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="60"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="15" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="B5" s="22" t="n">
+      <c r="B5" s="23" t="n">
         <v>2400000</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="19" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="19" t="s">
         <v>148</v>
       </c>
-      <c r="B6" s="23" t="n">
+      <c r="B6" s="24" t="n">
         <v>0.5</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="19" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="19" t="s">
         <v>150</v>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="23" t="n">
         <v>800000</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="19" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="19" t="s">
         <v>152</v>
       </c>
-      <c r="B8" s="22" t="n">
+      <c r="B8" s="23" t="n">
         <v>300000</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="19" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="22" t="s">
         <v>154</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="22" t="s">
         <v>155</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="22" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="B11" s="30" t="n">
+      <c r="B11" s="31" t="n">
         <f aca="false">$B$5</f>
         <v>2400000</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="19" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="19" t="s">
         <v>158</v>
       </c>
-      <c r="B12" s="30" t="n">
+      <c r="B12" s="31" t="n">
         <f aca="false">$B$5</f>
         <v>2400000</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="19" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="B13" s="30" t="n">
+      <c r="B13" s="31" t="n">
         <f aca="false">$B$5*$B$6</f>
         <v>1200000</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="19" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21" t="s">
         <v>105</v>
       </c>
-      <c r="B14" s="27" t="n">
+      <c r="B14" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="19" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="21" t="s">
         <v>163</v>
       </c>
-      <c r="B15" s="27" t="n">
+      <c r="B15" s="28" t="n">
         <f aca="false">$B$7</f>
         <v>800000</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="19" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="16" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="17" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="19" t="s">
         <v>166</v>
       </c>
-      <c r="B18" s="28" t="n">
+      <c r="B18" s="29" t="n">
         <f aca="false">IF($B$5=0,0,$B$7/$B$5)</f>
         <v>0.333333333333333</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="C18" s="19" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="18" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="B19" s="27" t="n">
+      <c r="B19" s="28" t="n">
         <f aca="false">B15+B8</f>
         <v>1100000</v>
       </c>
-      <c r="C19" s="18" t="s">
+      <c r="C19" s="19" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="18" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="27" t="n">
+      <c r="B20" s="28" t="n">
         <f aca="false">B11-B19</f>
         <v>1300000</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="C20" s="19" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="16" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="17" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="18" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="19" t="s">
         <v>171</v>
       </c>
-      <c r="B23" s="29" t="str">
+      <c r="B23" s="30" t="str">
         <f aca="false">IF(AND(B14&lt;=B15,B15&lt;=B13,B13&lt;=B12),"OK — ansvaret øker fra aksjeselskap via kausjon og DA til ANS og enkeltpersonforetak","AVVIK: sjekk eierandelen i B6 og kausjonen i B7 — stigen går ikke oppover")</f>
         <v>OK — ansvaret øker fra aksjeselskap via kausjon og DA til ANS og enkeltpersonforetak</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="18" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="19" t="s">
         <v>172</v>
       </c>
-      <c r="B24" s="29" t="str">
+      <c r="B24" s="30" t="str">
         <f aca="false">IF(B7&lt;=B5,"OK — kausjonen dekker en del av gjelden, ikke hele","AVVIK: en kausjon større enn den udekkede gjelden gir ikke mening her")</f>
         <v>OK — kausjonen dekker en del av gjelden, ikke hele</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="18" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="19" t="s">
         <v>173</v>
       </c>
-      <c r="B25" s="29" t="str">
+      <c r="B25" s="30" t="str">
         <f aca="false">IF(B20&gt;0,"OK — aksjeselskapet sparer deg for det beløpet som står i B20","AVVIK: med denne kausjonen er det ingenting igjen av ansvarsbegrensningen")</f>
         <v>OK — aksjeselskapet sparer deg for det beløpet som står i B20</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="20" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="21" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="16" t="s">
         <v>175</v>
       </c>
     </row>
@@ -2704,243 +2708,243 @@
   <dimension ref="A1:E30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="52"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="15" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="B5" s="22" t="n">
+      <c r="B5" s="23" t="n">
         <v>22400000</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="19" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="19" t="s">
         <v>181</v>
       </c>
-      <c r="B6" s="22" t="n">
-        <v>10200000</v>
-      </c>
-      <c r="E6" s="18" t="s">
+      <c r="B6" s="23" t="n">
+        <v>10182650</v>
+      </c>
+      <c r="E6" s="19" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="B7" s="31" t="n">
+      <c r="B7" s="32" t="n">
         <v>18</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="22" t="s">
         <v>184</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="22" t="s">
         <v>185</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="22" t="s">
         <v>186</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="D9" s="22" t="s">
         <v>187</v>
       </c>
-      <c r="E9" s="21" t="s">
+      <c r="E9" s="22" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="B10" s="26" t="n">
+      <c r="B10" s="27" t="n">
         <f aca="false">$B$5</f>
         <v>22400000</v>
       </c>
-      <c r="C10" s="22" t="n">
+      <c r="C10" s="23" t="n">
         <v>7000000</v>
       </c>
-      <c r="D10" s="19" t="str">
+      <c r="D10" s="20" t="str">
         <f aca="false">IF(B10&gt;C10,"JA — over grensen","Nei")</f>
         <v>JA — over grensen</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="E10" s="19" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="19" t="s">
         <v>191</v>
       </c>
-      <c r="B11" s="26" t="n">
+      <c r="B11" s="27" t="n">
         <f aca="false">$B$6</f>
-        <v>10200000</v>
-      </c>
-      <c r="C11" s="22" t="n">
+        <v>10182650</v>
+      </c>
+      <c r="C11" s="23" t="n">
         <v>27000000</v>
       </c>
-      <c r="D11" s="19" t="str">
+      <c r="D11" s="20" t="str">
         <f aca="false">IF(B11&gt;C11,"JA — over grensen","Nei")</f>
         <v>Nei</v>
       </c>
-      <c r="E11" s="18" t="s">
+      <c r="E11" s="19" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="B12" s="32" t="n">
+      <c r="B12" s="33" t="n">
         <f aca="false">$B$7</f>
         <v>18</v>
       </c>
-      <c r="C12" s="31" t="n">
+      <c r="C12" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="D12" s="19" t="str">
+      <c r="D12" s="20" t="str">
         <f aca="false">IF(B12&gt;C12,"JA — over grensen","Nei")</f>
         <v>JA — over grensen</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="E12" s="19" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="21" t="s">
         <v>195</v>
       </c>
-      <c r="B13" s="33" t="n">
+      <c r="B13" s="34" t="n">
         <f aca="false">COUNTIF(D10:D12,"JA*")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="16" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="17" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21" t="s">
         <v>105</v>
       </c>
-      <c r="D16" s="34" t="str">
+      <c r="D16" s="35" t="str">
         <f aca="false">IF(B13=0,"Kan velge bort revisor","Revisjonsplikt — minst én grense er passert")</f>
         <v>Revisjonsplikt — minst én grense er passert</v>
       </c>
-      <c r="E16" s="18" t="s">
+      <c r="E16" s="19" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="20" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="21" t="s">
         <v>198</v>
       </c>
-      <c r="D17" s="34" t="str">
+      <c r="D17" s="35" t="str">
         <f aca="false">IF(B13=0,"Fritatt for revisjon","Revisjonsplikt")</f>
         <v>Revisjonsplikt</v>
       </c>
-      <c r="E17" s="18" t="s">
+      <c r="E17" s="19" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="D18" s="20" t="s">
+      <c r="D18" s="21" t="s">
         <v>201</v>
       </c>
-      <c r="E18" s="18" t="s">
+      <c r="E18" s="19" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="16" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="17" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="18" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="19" t="s">
         <v>204</v>
       </c>
-      <c r="B21" s="22" t="n">
+      <c r="B21" s="23" t="n">
         <v>30000</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="18" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="19" t="s">
         <v>205</v>
       </c>
-      <c r="B22" s="22" t="n">
+      <c r="B22" s="23" t="n">
         <v>300000</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="18" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="19" t="s">
         <v>206</v>
       </c>
-      <c r="B23" s="35" t="n">
+      <c r="B23" s="36" t="n">
         <f aca="false">B22/B21</f>
         <v>10</v>
       </c>
-      <c r="E23" s="18" t="s">
+      <c r="E23" s="19" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="16" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="17" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="18" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="B26" s="29" t="str">
+      <c r="B26" s="30" t="str">
         <f aca="false">IF(B13&gt;0,"OK — bedriften har revisjonsplikt. Med Nordlys-tallene er den over på to av tre grenser: omsetning og årsverk","OK — bedriften er under alle tre grensene og kan velge bort revisor")</f>
         <v>OK — bedriften har revisjonsplikt. Med Nordlys-tallene er den over på to av tre grenser: omsetning og årsverk</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="18" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="19" t="s">
         <v>209</v>
       </c>
-      <c r="B27" s="29" t="str">
+      <c r="B27" s="30" t="str">
         <f aca="false">IF(B22&gt;=B21,"OK — aksjekapitalen er minst lovens minstekrav","AVVIK: aksjekapitalen er lavere enn minstekravet — et slikt aksjeselskap kan ikke registreres")</f>
         <v>OK — aksjekapitalen er minst lovens minstekrav</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="20" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="21" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="16" t="s">
         <v>211</v>
       </c>
     </row>
@@ -2973,528 +2977,528 @@
   <dimension ref="A1:E67"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="54"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="15" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21"/>
-      <c r="B7" s="21" t="s">
+      <c r="A7" s="22"/>
+      <c r="B7" s="22" t="s">
         <v>216</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="22" t="s">
         <v>217</v>
       </c>
-      <c r="D7" s="21" t="s">
+      <c r="D7" s="22" t="s">
         <v>218</v>
       </c>
-      <c r="E7" s="21" t="s">
+      <c r="E7" s="22" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="B8" s="22" t="n">
+      <c r="B8" s="23" t="n">
         <v>300000</v>
       </c>
-      <c r="C8" s="30" t="n">
+      <c r="C8" s="31" t="n">
         <f aca="false">Skatt!B5</f>
         <v>900000</v>
       </c>
-      <c r="D8" s="22" t="n">
+      <c r="D8" s="23" t="n">
         <v>1800000</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="E8" s="19" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="19" t="s">
         <v>221</v>
       </c>
-      <c r="B9" s="26" t="n">
+      <c r="B9" s="27" t="n">
         <f aca="false">B8*(1-Skatt!$B$6)</f>
         <v>198000</v>
       </c>
-      <c r="C9" s="26" t="n">
+      <c r="C9" s="27" t="n">
         <f aca="false">C8*(1-Skatt!$B$6)</f>
         <v>594000</v>
       </c>
-      <c r="D9" s="26" t="n">
+      <c r="D9" s="27" t="n">
         <f aca="false">D8*(1-Skatt!$B$6)</f>
         <v>1188000</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="19" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="19" t="s">
         <v>223</v>
       </c>
-      <c r="B10" s="26" t="n">
+      <c r="B10" s="27" t="n">
         <f aca="false">B8*(1-Skatt!$B$7)</f>
         <v>234000</v>
       </c>
-      <c r="C10" s="26" t="n">
+      <c r="C10" s="27" t="n">
         <f aca="false">C8*(1-Skatt!$B$7)</f>
         <v>702000</v>
       </c>
-      <c r="D10" s="26" t="n">
+      <c r="D10" s="27" t="n">
         <f aca="false">D8*(1-Skatt!$B$7)</f>
         <v>1404000</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="E10" s="19" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="19" t="s">
         <v>225</v>
       </c>
-      <c r="B11" s="26" t="n">
+      <c r="B11" s="27" t="n">
         <f aca="false">B10*(1-Skatt!$B$9)</f>
         <v>145454.4</v>
       </c>
-      <c r="C11" s="26" t="n">
+      <c r="C11" s="27" t="n">
         <f aca="false">C10*(1-Skatt!$B$9)</f>
         <v>436363.2</v>
       </c>
-      <c r="D11" s="26" t="n">
+      <c r="D11" s="27" t="n">
         <f aca="false">D10*(1-Skatt!$B$9)</f>
         <v>872726.4</v>
       </c>
-      <c r="E11" s="18" t="s">
+      <c r="E11" s="19" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21" t="s">
         <v>227</v>
       </c>
-      <c r="B12" s="27" t="n">
+      <c r="B12" s="28" t="n">
         <f aca="false">B10-B9</f>
         <v>36000</v>
       </c>
-      <c r="C12" s="27" t="n">
+      <c r="C12" s="28" t="n">
         <f aca="false">C10-C9</f>
         <v>108000</v>
       </c>
-      <c r="D12" s="27" t="n">
+      <c r="D12" s="28" t="n">
         <f aca="false">D10-D9</f>
         <v>216000</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="E12" s="19" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="21" t="s">
         <v>229</v>
       </c>
-      <c r="B13" s="27" t="n">
+      <c r="B13" s="28" t="n">
         <f aca="false">B11-B9</f>
         <v>-52545.6</v>
       </c>
-      <c r="C13" s="27" t="n">
+      <c r="C13" s="28" t="n">
         <f aca="false">C11-C9</f>
         <v>-157636.8</v>
       </c>
-      <c r="D13" s="27" t="n">
+      <c r="D13" s="28" t="n">
         <f aca="false">D11-D9</f>
         <v>-315273.6</v>
       </c>
-      <c r="E13" s="18" t="s">
+      <c r="E13" s="19" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="18" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="19" t="s">
         <v>231</v>
       </c>
-      <c r="B14" s="36" t="n">
+      <c r="B14" s="37" t="n">
         <f aca="false">B12/B8</f>
         <v>0.12</v>
       </c>
-      <c r="C14" s="36" t="n">
+      <c r="C14" s="37" t="n">
         <f aca="false">C12/C8</f>
         <v>0.12</v>
       </c>
-      <c r="D14" s="36" t="n">
+      <c r="D14" s="37" t="n">
         <f aca="false">D12/D8</f>
         <v>0.12</v>
       </c>
-      <c r="E14" s="18" t="s">
+      <c r="E14" s="19" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="16" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="17" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="19" t="s">
         <v>233</v>
       </c>
-      <c r="B17" s="29" t="str">
+      <c r="B17" s="30" t="str">
         <f aca="false">IF(AND(ABS(B14-C14)&lt;0.0001,ABS(C14-D14)&lt;0.0001),"OK — samme prosent på alle tre nivåene. Skatten skalerer, og derfor blir den aldri det avgjørende argumentet","AVVIK: satsene er ikke flate — sjekk Skatt!B6, B7 og B8")</f>
         <v>OK — samme prosent på alle tre nivåene. Skatten skalerer, og derfor blir den aldri det avgjørende argumentet</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="16" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="17" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="15" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="16" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="18" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="B23" s="26" t="n">
+      <c r="B23" s="27" t="n">
         <f aca="false">Ansvar!B5</f>
         <v>2400000</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="18" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="19" t="s">
         <v>236</v>
       </c>
-      <c r="B24" s="30" t="n">
+      <c r="B24" s="31" t="n">
         <f aca="false">Ansvar!B11</f>
         <v>2400000</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="18" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="19" t="s">
         <v>237</v>
       </c>
-      <c r="B25" s="30" t="n">
+      <c r="B25" s="31" t="n">
         <f aca="false">Ansvar!B15+Ansvar!B8</f>
         <v>1100000</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="20" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="B26" s="27" t="n">
+      <c r="B26" s="28" t="n">
         <f aca="false">B24-B25</f>
         <v>1300000</v>
       </c>
-      <c r="E26" s="18" t="s">
+      <c r="E26" s="19" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="18" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="19" t="s">
         <v>240</v>
       </c>
-      <c r="B27" s="26" t="n">
+      <c r="B27" s="27" t="n">
         <f aca="false">Skatt!B20</f>
         <v>594000</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="20" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="21" t="s">
         <v>241</v>
       </c>
-      <c r="B28" s="37" t="n">
+      <c r="B28" s="38" t="n">
         <f aca="false">B26/B27</f>
         <v>2.18855218855219</v>
       </c>
-      <c r="E28" s="18" t="s">
+      <c r="E28" s="19" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="18" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="B29" s="22" t="n">
+      <c r="B29" s="23" t="n">
         <v>25000</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="18" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="19" t="s">
         <v>244</v>
       </c>
-      <c r="B30" s="35" t="n">
+      <c r="B30" s="36" t="n">
         <f aca="false">IF(B29=0,0,B26/B29)</f>
         <v>52</v>
       </c>
-      <c r="E30" s="18" t="s">
+      <c r="E30" s="19" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="16" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="17" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="18" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="19" t="s">
         <v>246</v>
       </c>
-      <c r="B33" s="29" t="str">
+      <c r="B33" s="30" t="str">
         <f aca="false">IF(B30&gt;10,"OK — det tar mer enn ti år med merkostnad før aksjeselskapet er like dyrt som én konkurs. Det er derfor ansvaret veier tyngre enn skatten","AVVIK: her er merkostnaden så høy at regnestykket bør gjøres på nytt")</f>
         <v>OK — det tar mer enn ti år med merkostnad før aksjeselskapet er like dyrt som én konkurs. Det er derfor ansvaret veier tyngre enn skatten</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="16" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="17" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="15" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="16" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="15" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="16" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="18" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="19" t="s">
         <v>250</v>
       </c>
-      <c r="B39" s="31" t="n">
+      <c r="B39" s="32" t="n">
         <v>1102</v>
       </c>
-      <c r="E39" s="18" t="s">
+      <c r="E39" s="19" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="18" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="19" t="s">
         <v>252</v>
       </c>
-      <c r="B40" s="38" t="n">
+      <c r="B40" s="39" t="n">
         <v>890</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="18" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="19" t="s">
         <v>253</v>
       </c>
-      <c r="B41" s="27" t="n">
+      <c r="B41" s="28" t="n">
         <f aca="false">B39*B40</f>
         <v>980780</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="18" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="19" t="s">
         <v>254</v>
       </c>
-      <c r="B42" s="22" t="n">
+      <c r="B42" s="23" t="n">
         <v>133111.111111111</v>
       </c>
-      <c r="E42" s="18" t="s">
+      <c r="E42" s="19" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="18" t="s">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="19" t="s">
         <v>256</v>
       </c>
-      <c r="B43" s="22" t="n">
+      <c r="B43" s="23" t="n">
         <v>260000</v>
       </c>
-      <c r="E43" s="18" t="s">
+      <c r="E43" s="19" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="20" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="21" t="s">
         <v>258</v>
       </c>
-      <c r="B44" s="27" t="n">
+      <c r="B44" s="28" t="n">
         <f aca="false">B41+B42-B43</f>
         <v>853891.111111111</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="16" t="s">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="17" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="18" t="s">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="19" t="s">
         <v>260</v>
       </c>
-      <c r="B47" s="30" t="n">
+      <c r="B47" s="31" t="n">
         <f aca="false">B44*(1-Skatt!$B$6)</f>
         <v>563568.133333333</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="18" t="s">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="19" t="s">
         <v>261</v>
       </c>
-      <c r="B48" s="30" t="n">
+      <c r="B48" s="31" t="n">
         <f aca="false">B44*(1-Skatt!$B$7)</f>
         <v>666035.066666667</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="18" t="s">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="19" t="s">
         <v>225</v>
       </c>
-      <c r="B49" s="30" t="n">
+      <c r="B49" s="31" t="n">
         <f aca="false">B48*(1-Skatt!$B$9)</f>
         <v>414007.39744</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="20" t="s">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="21" t="s">
         <v>262</v>
       </c>
-      <c r="B50" s="27" t="n">
+      <c r="B50" s="28" t="n">
         <f aca="false">B48-B47</f>
         <v>102466.933333333</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="20" t="s">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="21" t="s">
         <v>263</v>
       </c>
-      <c r="B51" s="27" t="n">
+      <c r="B51" s="28" t="n">
         <f aca="false">B49-B47</f>
         <v>-149560.735893333</v>
       </c>
-      <c r="E51" s="18" t="s">
+      <c r="E51" s="19" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="18" t="s">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="B52" s="26" t="n">
+      <c r="B52" s="27" t="n">
         <f aca="false">B29</f>
         <v>25000</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="20" t="s">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="21" t="s">
         <v>265</v>
       </c>
-      <c r="B53" s="27" t="n">
+      <c r="B53" s="28" t="n">
         <f aca="false">B50-B52</f>
         <v>77466.9333333335</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="18" t="s">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="19" t="s">
         <v>266</v>
       </c>
-      <c r="B54" s="35" t="n">
+      <c r="B54" s="36" t="n">
         <f aca="false">B52/B40</f>
         <v>28.0898876404494</v>
       </c>
-      <c r="E54" s="18" t="s">
+      <c r="E54" s="19" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="16" t="s">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="17" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="18" t="s">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="19" t="s">
         <v>269</v>
       </c>
-      <c r="B57" s="22" t="n">
+      <c r="B57" s="23" t="n">
         <v>2400000</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="20" t="s">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="21" t="s">
         <v>270</v>
       </c>
-      <c r="B58" s="37" t="n">
+      <c r="B58" s="38" t="n">
         <f aca="false">B57/B47</f>
         <v>4.25858003326897</v>
       </c>
-      <c r="E58" s="18" t="s">
+      <c r="E58" s="19" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="16" t="s">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="17" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="18" t="s">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="19" t="s">
         <v>272</v>
       </c>
-      <c r="B61" s="29" t="str">
+      <c r="B61" s="30" t="str">
         <f aca="false">IF(B51&lt;0,"AVVIK: skattefordelen er negativ — aksjeselskap koster ham penger på skatten når han tar ut hele overskuddet","OK — skatten taler for aksjeselskap også ved fullt uttak")</f>
         <v>AVVIK: skattefordelen er negativ — aksjeselskap koster ham penger på skatten når han tar ut hele overskuddet</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="15" t="s">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="16" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="18" t="s">
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="19" t="s">
         <v>274</v>
       </c>
-      <c r="B63" s="29" t="str">
+      <c r="B63" s="30" t="str">
         <f aca="false">IF(B41+B42&lt;Grenser!C10,"OK — han er under grensen for driftsinntekter og kan velge bort revisor det første året","AVVIK: han passerer revisjonsgrensen allerede første år")</f>
         <v>OK — han er under grensen for driftsinntekter og kan velge bort revisor det første året</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="18" t="s">
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="19" t="s">
         <v>275</v>
       </c>
-      <c r="B64" s="29" t="str">
+      <c r="B64" s="30" t="str">
         <f aca="false">IF(B58&gt;2,"OK — ansvarssaken tilsvarer mer enn to års inntekt etter skatt. Det er derfor ansvaret veier tyngre enn skatten i denne drøftingen","AVVIK: med disse tallene er ansvarsrisikoen for liten til å bære drøftingen")</f>
         <v>OK — ansvarssaken tilsvarer mer enn to års inntekt etter skatt. Det er derfor ansvaret veier tyngre enn skatten i denne drøftingen</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="15" t="s">
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="16" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="15" t="s">
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="16" t="s">
         <v>90</v>
       </c>
     </row>

</xml_diff>